<commit_message>
Added User Stories and updated Part 2 excel document
</commit_message>
<xml_diff>
--- a/Milestone 1/Milestone 1 - Part 2.xlsx
+++ b/Milestone 1/Milestone 1 - Part 2.xlsx
@@ -5,16 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jus10albeck/Desktop/School/GCU/CST-326 Written and Verbal Communication for SD /Topic 2 /"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jus10albeck/Desktop/School/GCU/CST-326 Written and Verbal Communication for SD /CST-326 Milestone Project/Milestone 1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95F89154-A8DB-C44C-99CE-3ED996D4EE93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A82CAD4B-103F-E04D-AA7B-E65A8DFFD846}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39300" yWindow="820" windowWidth="27180" windowHeight="20780" activeTab="1" xr2:uid="{96A73B82-89FE-E94A-AC13-DCA1005713DC}"/>
+    <workbookView xWindow="38560" yWindow="660" windowWidth="29300" windowHeight="20780" activeTab="2" xr2:uid="{96A73B82-89FE-E94A-AC13-DCA1005713DC}"/>
   </bookViews>
   <sheets>
     <sheet name="Questions" sheetId="1" r:id="rId1"/>
     <sheet name="Responses" sheetId="2" r:id="rId2"/>
+    <sheet name="Backlog Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="190">
   <si>
     <t>ID</t>
   </si>
@@ -359,6 +360,282 @@
   </si>
   <si>
     <t>under repair, lost, reserverd, retired</t>
+  </si>
+  <si>
+    <t>Devin Puckett</t>
+  </si>
+  <si>
+    <t>Name, category, serial number, location, condition, status</t>
+  </si>
+  <si>
+    <t>Name, category, serial number, status</t>
+  </si>
+  <si>
+    <t>Under repair, lost, reserved, retired</t>
+  </si>
+  <si>
+    <t>Story</t>
+  </si>
+  <si>
+    <t>Feature Area</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>US-1</t>
+  </si>
+  <si>
+    <t>US-2</t>
+  </si>
+  <si>
+    <t>US-3</t>
+  </si>
+  <si>
+    <t>US-4</t>
+  </si>
+  <si>
+    <t>US-5</t>
+  </si>
+  <si>
+    <t>US-6</t>
+  </si>
+  <si>
+    <t>US-7</t>
+  </si>
+  <si>
+    <t>US-8</t>
+  </si>
+  <si>
+    <t>US-9</t>
+  </si>
+  <si>
+    <t>US-10</t>
+  </si>
+  <si>
+    <t>US-11</t>
+  </si>
+  <si>
+    <t>US-12</t>
+  </si>
+  <si>
+    <t>US-13</t>
+  </si>
+  <si>
+    <t>US-14</t>
+  </si>
+  <si>
+    <t>US-15</t>
+  </si>
+  <si>
+    <t>US-16</t>
+  </si>
+  <si>
+    <t>US-17</t>
+  </si>
+  <si>
+    <t>US-18</t>
+  </si>
+  <si>
+    <t>US-19</t>
+  </si>
+  <si>
+    <t>US-20</t>
+  </si>
+  <si>
+    <t>US-21</t>
+  </si>
+  <si>
+    <t>US-22</t>
+  </si>
+  <si>
+    <t>US-23</t>
+  </si>
+  <si>
+    <t>US-24</t>
+  </si>
+  <si>
+    <t>US-25</t>
+  </si>
+  <si>
+    <t>US-26</t>
+  </si>
+  <si>
+    <t>US-27</t>
+  </si>
+  <si>
+    <t>US-28</t>
+  </si>
+  <si>
+    <t>US-29</t>
+  </si>
+  <si>
+    <t>US-30</t>
+  </si>
+  <si>
+    <t>US-31</t>
+  </si>
+  <si>
+    <t>US-32</t>
+  </si>
+  <si>
+    <t>US-33</t>
+  </si>
+  <si>
+    <t>US-34</t>
+  </si>
+  <si>
+    <t>US-35</t>
+  </si>
+  <si>
+    <t>US-36</t>
+  </si>
+  <si>
+    <t>Log in</t>
+  </si>
+  <si>
+    <t>Accounts and Access</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Admin creates accounts</t>
+  </si>
+  <si>
+    <t>Role-based permissions</t>
+  </si>
+  <si>
+    <t>Admin resets password</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Deactivate account</t>
+  </si>
+  <si>
+    <t>Self sign-up with approval</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Add equipment</t>
+  </si>
+  <si>
+    <t>Equipment Management (Administrator)</t>
+  </si>
+  <si>
+    <t>Edit equipment</t>
+  </si>
+  <si>
+    <t>Retire equipment</t>
+  </si>
+  <si>
+    <t>Change equipment status</t>
+  </si>
+  <si>
+    <t>Upload photo</t>
+  </si>
+  <si>
+    <t>Manage categories</t>
+  </si>
+  <si>
+    <t>View equipment list</t>
+  </si>
+  <si>
+    <t>Browsing and Search</t>
+  </si>
+  <si>
+    <t>View item details</t>
+  </si>
+  <si>
+    <t>Search equipment</t>
+  </si>
+  <si>
+    <t>Filter equipment</t>
+  </si>
+  <si>
+    <t>See units available per model</t>
+  </si>
+  <si>
+    <t>Check out equipment</t>
+  </si>
+  <si>
+    <t>Checkout and Return</t>
+  </si>
+  <si>
+    <t>Return equipment</t>
+  </si>
+  <si>
+    <t>See due dates</t>
+  </si>
+  <si>
+    <t>Admin records a return</t>
+  </si>
+  <si>
+    <t>Checkout limit</t>
+  </si>
+  <si>
+    <t>Request a reservation</t>
+  </si>
+  <si>
+    <t>Reservations</t>
+  </si>
+  <si>
+    <t>Approve or deny reservations</t>
+  </si>
+  <si>
+    <t>View my reservations</t>
+  </si>
+  <si>
+    <t>My current equipment</t>
+  </si>
+  <si>
+    <t>History</t>
+  </si>
+  <si>
+    <t>My checkout history</t>
+  </si>
+  <si>
+    <t>Item history</t>
+  </si>
+  <si>
+    <t>Report damaged equipment</t>
+  </si>
+  <si>
+    <t>Damage Reports</t>
+  </si>
+  <si>
+    <t>Review damage reports</t>
+  </si>
+  <si>
+    <t>Overdue reminder</t>
+  </si>
+  <si>
+    <t>Notifications</t>
+  </si>
+  <si>
+    <t>Reservation notification</t>
+  </si>
+  <si>
+    <t>Printable notices</t>
+  </si>
+  <si>
+    <t>Summary page</t>
+  </si>
+  <si>
+    <t>Administrator Dashboard</t>
+  </si>
+  <si>
+    <t>Overdue list</t>
+  </si>
+  <si>
+    <t>Mobile-friendly layout</t>
+  </si>
+  <si>
+    <t>Devices</t>
   </si>
 </sst>
 </file>
@@ -413,7 +690,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -483,11 +760,57 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -520,7 +843,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -532,11 +855,90 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -867,7 +1269,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9782D891-2DC3-5449-A7B1-599A4F2E29DC}">
   <dimension ref="A1:D22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="32.1640625" style="4" customWidth="1"/>
@@ -1192,11 +1594,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B1A6FCA-F0CB-3C4B-9EB0-0E65F0D39EDA}">
   <dimension ref="A1:C73"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.5" customWidth="1"/>
     <col min="2" max="2" width="8.33203125" style="4" customWidth="1"/>
-    <col min="3" max="3" width="21.1640625" style="11" customWidth="1"/>
+    <col min="3" max="3" width="47" style="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -1219,7 +1621,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="9" t="s">
         <v>72</v>
       </c>
@@ -1272,7 +1674,7 @@
         <v>78</v>
       </c>
       <c r="C10" s="14">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -1307,7 +1709,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B15" s="9" t="s">
         <v>83</v>
       </c>
@@ -1320,7 +1722,7 @@
         <v>84</v>
       </c>
       <c r="C16" s="14">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -1388,20 +1790,22 @@
       </c>
     </row>
     <row r="26" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A27" s="6">
         <v>2</v>
       </c>
       <c r="B27" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="C27" s="12"/>
+      <c r="C27" s="16" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="28" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B28" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C28" s="13" t="s">
+      <c r="C28" s="17" t="s">
         <v>93</v>
       </c>
     </row>
@@ -1409,127 +1813,169 @@
       <c r="B29" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C29" s="14"/>
+      <c r="C29" s="18" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B30" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C30" s="14"/>
+      <c r="C30" s="19">
+        <v>1</v>
+      </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B31" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="C31" s="14"/>
+      <c r="C31" s="19">
+        <v>3</v>
+      </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B32" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="C32" s="14"/>
+      <c r="C32" s="19">
+        <v>1</v>
+      </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B33" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C33" s="14"/>
+      <c r="C33" s="19">
+        <v>2</v>
+      </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B34" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="C34" s="14"/>
+      <c r="C34" s="18" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B35" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="C35" s="14"/>
+      <c r="C35" s="19">
+        <v>2</v>
+      </c>
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B36" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="C36" s="14"/>
+      <c r="C36" s="19">
+        <v>1</v>
+      </c>
     </row>
     <row r="37" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B37" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="C37" s="14"/>
+      <c r="C37" s="19">
+        <v>1</v>
+      </c>
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B38" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="C38" s="14"/>
+      <c r="C38" s="19">
+        <v>2</v>
+      </c>
     </row>
     <row r="39" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B39" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="C39" s="14"/>
+      <c r="C39" s="19">
+        <v>2</v>
+      </c>
     </row>
     <row r="40" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B40" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="C40" s="14"/>
+      <c r="C40" s="18" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B41" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="C41" s="14"/>
+      <c r="C41" s="19">
+        <v>1</v>
+      </c>
     </row>
     <row r="42" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B42" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="C42" s="14"/>
+      <c r="C42" s="19">
+        <v>2</v>
+      </c>
     </row>
     <row r="43" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B43" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="C43" s="14"/>
+      <c r="C43" s="20">
+        <v>2</v>
+      </c>
     </row>
     <row r="44" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B44" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="C44" s="14"/>
+      <c r="C44" s="19">
+        <v>2</v>
+      </c>
     </row>
     <row r="45" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B45" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="C45" s="14"/>
+      <c r="C45" s="19">
+        <v>1</v>
+      </c>
     </row>
     <row r="46" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B46" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C46" s="14"/>
+      <c r="C46" s="19">
+        <v>2</v>
+      </c>
     </row>
     <row r="47" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B47" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C47" s="14"/>
+      <c r="C47" s="19">
+        <v>2</v>
+      </c>
     </row>
     <row r="48" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B48" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="C48" s="14"/>
+      <c r="C48" s="19">
+        <v>2</v>
+      </c>
     </row>
     <row r="49" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B49" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="C49" s="15"/>
+      <c r="C49" s="21">
+        <v>2</v>
+      </c>
     </row>
     <row r="50" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
@@ -1679,4 +2125,549 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4404C535-C6DD-8E44-AF8D-B98D5170B1BC}">
+  <dimension ref="B2:E38"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="7.33203125" customWidth="1"/>
+    <col min="3" max="3" width="32.6640625" customWidth="1"/>
+    <col min="4" max="4" width="37.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B2" s="22" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="22" t="s">
+        <v>102</v>
+      </c>
+      <c r="D2" s="22" t="s">
+        <v>103</v>
+      </c>
+      <c r="E2" s="22" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="23" t="s">
+        <v>105</v>
+      </c>
+      <c r="C3" s="23" t="s">
+        <v>141</v>
+      </c>
+      <c r="D3" s="23" t="s">
+        <v>142</v>
+      </c>
+      <c r="E3" s="23" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B4" s="23" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="23" t="s">
+        <v>144</v>
+      </c>
+      <c r="D4" s="23" t="s">
+        <v>142</v>
+      </c>
+      <c r="E4" s="23" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="23" t="s">
+        <v>107</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>145</v>
+      </c>
+      <c r="D5" s="23" t="s">
+        <v>142</v>
+      </c>
+      <c r="E5" s="23" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B6" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="C6" s="23" t="s">
+        <v>146</v>
+      </c>
+      <c r="D6" s="23" t="s">
+        <v>142</v>
+      </c>
+      <c r="E6" s="23" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B7" s="23" t="s">
+        <v>109</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>142</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="23" t="s">
+        <v>110</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>149</v>
+      </c>
+      <c r="D8" s="23" t="s">
+        <v>142</v>
+      </c>
+      <c r="E8" s="23" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="23" t="s">
+        <v>111</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="D9" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="E9" s="23" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="D10" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="E10" s="23" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="23" t="s">
+        <v>113</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="D11" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="E11" s="23" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="23" t="s">
+        <v>114</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>155</v>
+      </c>
+      <c r="D12" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="E12" s="23" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="C13" s="23" t="s">
+        <v>156</v>
+      </c>
+      <c r="D13" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="E13" s="23" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="23" t="s">
+        <v>116</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>157</v>
+      </c>
+      <c r="D14" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="E14" s="23" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="C15" s="23" t="s">
+        <v>158</v>
+      </c>
+      <c r="D15" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="E15" s="23" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="23" t="s">
+        <v>118</v>
+      </c>
+      <c r="C16" s="23" t="s">
+        <v>160</v>
+      </c>
+      <c r="D16" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="E16" s="23" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="23" t="s">
+        <v>119</v>
+      </c>
+      <c r="C17" s="23" t="s">
+        <v>161</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="E17" s="23" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="C18" s="23" t="s">
+        <v>162</v>
+      </c>
+      <c r="D18" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="E18" s="23" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="23" t="s">
+        <v>121</v>
+      </c>
+      <c r="C19" s="23" t="s">
+        <v>163</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="E19" s="23" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="23" t="s">
+        <v>122</v>
+      </c>
+      <c r="C20" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="E20" s="23" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="23" t="s">
+        <v>123</v>
+      </c>
+      <c r="C21" s="23" t="s">
+        <v>166</v>
+      </c>
+      <c r="D21" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="E21" s="23" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="23" t="s">
+        <v>124</v>
+      </c>
+      <c r="C22" s="23" t="s">
+        <v>167</v>
+      </c>
+      <c r="D22" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="E22" s="23" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="C23" s="23" t="s">
+        <v>168</v>
+      </c>
+      <c r="D23" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="E23" s="23" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B24" s="23" t="s">
+        <v>126</v>
+      </c>
+      <c r="C24" s="23" t="s">
+        <v>169</v>
+      </c>
+      <c r="D24" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="E24" s="23" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="C25" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="D25" s="23" t="s">
+        <v>171</v>
+      </c>
+      <c r="E25" s="23" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B26" s="23" t="s">
+        <v>128</v>
+      </c>
+      <c r="C26" s="23" t="s">
+        <v>172</v>
+      </c>
+      <c r="D26" s="23" t="s">
+        <v>171</v>
+      </c>
+      <c r="E26" s="23" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B27" s="23" t="s">
+        <v>129</v>
+      </c>
+      <c r="C27" s="23" t="s">
+        <v>173</v>
+      </c>
+      <c r="D27" s="23" t="s">
+        <v>171</v>
+      </c>
+      <c r="E27" s="23" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B28" s="23" t="s">
+        <v>130</v>
+      </c>
+      <c r="C28" s="23" t="s">
+        <v>174</v>
+      </c>
+      <c r="D28" s="23" t="s">
+        <v>175</v>
+      </c>
+      <c r="E28" s="23" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B29" s="23" t="s">
+        <v>131</v>
+      </c>
+      <c r="C29" s="23" t="s">
+        <v>176</v>
+      </c>
+      <c r="D29" s="23" t="s">
+        <v>175</v>
+      </c>
+      <c r="E29" s="23" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B30" s="23" t="s">
+        <v>132</v>
+      </c>
+      <c r="C30" s="23" t="s">
+        <v>177</v>
+      </c>
+      <c r="D30" s="23" t="s">
+        <v>175</v>
+      </c>
+      <c r="E30" s="23" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B31" s="23" t="s">
+        <v>133</v>
+      </c>
+      <c r="C31" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="D31" s="23" t="s">
+        <v>179</v>
+      </c>
+      <c r="E31" s="23" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B32" s="23" t="s">
+        <v>134</v>
+      </c>
+      <c r="C32" s="23" t="s">
+        <v>180</v>
+      </c>
+      <c r="D32" s="23" t="s">
+        <v>179</v>
+      </c>
+      <c r="E32" s="23" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B33" s="23" t="s">
+        <v>135</v>
+      </c>
+      <c r="C33" s="23" t="s">
+        <v>181</v>
+      </c>
+      <c r="D33" s="23" t="s">
+        <v>182</v>
+      </c>
+      <c r="E33" s="23" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B34" s="23" t="s">
+        <v>136</v>
+      </c>
+      <c r="C34" s="23" t="s">
+        <v>183</v>
+      </c>
+      <c r="D34" s="23" t="s">
+        <v>182</v>
+      </c>
+      <c r="E34" s="23" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B35" s="23" t="s">
+        <v>137</v>
+      </c>
+      <c r="C35" s="23" t="s">
+        <v>184</v>
+      </c>
+      <c r="D35" s="23" t="s">
+        <v>182</v>
+      </c>
+      <c r="E35" s="23" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B36" s="23" t="s">
+        <v>138</v>
+      </c>
+      <c r="C36" s="23" t="s">
+        <v>185</v>
+      </c>
+      <c r="D36" s="23" t="s">
+        <v>186</v>
+      </c>
+      <c r="E36" s="23" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="37" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B37" s="23" t="s">
+        <v>139</v>
+      </c>
+      <c r="C37" s="23" t="s">
+        <v>187</v>
+      </c>
+      <c r="D37" s="23" t="s">
+        <v>186</v>
+      </c>
+      <c r="E37" s="23" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="38" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B38" s="23" t="s">
+        <v>140</v>
+      </c>
+      <c r="C38" s="23" t="s">
+        <v>188</v>
+      </c>
+      <c r="D38" s="23" t="s">
+        <v>189</v>
+      </c>
+      <c r="E38" s="23" t="s">
+        <v>150</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <conditionalFormatting sqref="E1:E1048576">
+    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="High">
+      <formula>NOT(ISERROR(SEARCH("High",E1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Medium">
+      <formula>NOT(ISERROR(SEARCH("Medium",E1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Low">
+      <formula>NOT(ISERROR(SEARCH("Low",E1)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>